<commit_message>
Leads: 2026-10-07 15:25 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-07.xlsx
+++ b/output/leads_2026-10-07.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,66 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Plumbing Contractor Cambridge, MA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>kirklandandshaw.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://www.kirklandandshaw.com/plumbing-contractor-cambridge-ma</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Heating Experience</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>office@kirklandandshaw.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>(781) 272-2670</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Cambridge MA</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>90</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>plumbing company Cambridge MA</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-07 15:29 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-07.xlsx
+++ b/output/leads_2026-10-07.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -623,6 +623,66 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Aaron's Plumbing</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>aaronsplumbingmi.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://aaronsplumbingmi.com/</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Recent Hints</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>aarons.plumbing@outlook.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>517-321-8700</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Lansing MI</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>96</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>plumber Lansing MI</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-07 15:30 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-07.xlsx
+++ b/output/leads_2026-10-07.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -683,6 +683,66 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Action Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>actionairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://actionairconditioning.com/service-area/clearwater/ac-repair/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Action Air</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>info@actionairconditioning.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(813) 935-6644</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Clearwater FL</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>air conditioning repair Clearwater FL</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-07 15:32 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-07.xlsx
+++ b/output/leads_2026-10-07.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -743,6 +743,66 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation in Lowell</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>forgeco.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://www.forgeco.com/locality/lowell</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Mark Kasdorf</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>hello@forgeco.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>617-546-7004</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Lowell MA</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>88</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>heat pump installation Lowell MA</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-07 15:35 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-07.xlsx
+++ b/output/leads_2026-10-07.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -803,6 +803,62 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Metal Roof Indianapolis</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>metalroofindianapolis.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>http://www.metalroofindianapolis.com/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>moreinfo@metalroofindianapolis.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>317-383-0645</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Indianapolis IN</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>84</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Indianapolis IN</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-07 15:37 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-07.xlsx
+++ b/output/leads_2026-10-07.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -824,7 +824,6 @@
           <t>http://www.metalroofindianapolis.com/</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>moreinfo@metalroofindianapolis.com</t>
@@ -854,6 +853,182 @@
         </is>
       </c>
       <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Heating &amp; AC Repair Greater Kansas City | Dyno Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>hvacdyno.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://www.hvacdyno.com/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Across Kansas</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>dynohvac10@gmail.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>026-0012422</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Kansas City KS</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>90</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>heating and cooling company Kansas City KS</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Plumber in San Marcos | Copperfield Plumbing Services</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>copperfieldplumbingservices.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://www.copperfieldplumbingservices.com/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Copperfield Plumbing</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>info@copperfieldplumbingservices.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(512) 667-6776</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>San Marcos TX</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>90</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>plumber San Marcos TX</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Koch Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>kochheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://kochheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>kochhvacinc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(913) 287-9055</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Kansas City KS</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>88</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>heating and cooling company Kansas City KS</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-07 21:08 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-07.xlsx
+++ b/output/leads_2026-10-07.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -999,7 +999,6 @@
           <t>https://kochheatingandcooling.com/</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>kochhvacinc@gmail.com</t>
@@ -1029,6 +1028,126 @@
         </is>
       </c>
       <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>YHS â Your Home Solutions, Inc.</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>yhsillinois.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://yhsillinois.com/roofing-elgin-il</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Mission Every</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>info@yhsillinois.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(888) 470-9474</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Elgin IL</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>90</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>roofing contractor Elgin IL</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Cool AC Services</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>coolacservices.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://coolacservices.com/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Homeowners Trust</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>ceo@coolacservices.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(727) 315-0793</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Clearwater FL</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>90</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>heating and cooling company Clearwater FL</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-07 21:09 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-07.xlsx
+++ b/output/leads_2026-10-07.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1153,6 +1153,126 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Terry Vereen Plumbing</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>terryvereenplumbing.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.terryvereenplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Duval County</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>ar@terryvereenplumbing.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>904-384-5661</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>90</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>plumbing company Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>North Florida Plumbing LLC</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>northfloridaplumbing.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.northfloridaplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>James Conner</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>jamesconnernfp@gmail.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(904) 862-6927</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>90</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>plumbing company Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-07 21:14 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-07.xlsx
+++ b/output/leads_2026-10-07.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1273,6 +1273,126 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Paramount Roofing &amp; Consulting</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>paramountroofingandconsulting.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.paramountroofingandconsulting.com/service-areas/roswell-ga/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Storm Damage</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>info@paramountroofingandconsulting.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(404) 971-2880</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Roswell GA</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>roof repair company Roswell GA</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Plumber in El Paso, TX | Licensed Pros</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>joesplumber.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://joesplumber.com/tx/el-paso/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>El Paso</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>info@joesplumber.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(207) 419-2600</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>El Paso TX</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>90</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>plumber El Paso TX</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-07 21:21 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-07.xlsx
+++ b/output/leads_2026-10-07.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1393,6 +1393,62 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Absolute Services</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>absoluteservices803.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://absoluteservices803.com/heating-repair</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>micah@micahrich.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>(803) 708-1664</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Columbia SC</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>80</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>furnace repair Columbia SC</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-07 21:24 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-07.xlsx
+++ b/output/leads_2026-10-07.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1414,7 +1414,6 @@
           <t>https://absoluteservices803.com/heating-repair</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>micah@micahrich.com</t>
@@ -1444,6 +1443,66 @@
         </is>
       </c>
       <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Forefront</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>forefrontroofinginc.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://www.forefrontroofinginc.com/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Southern California</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>info@forefrontroofinginc.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>800-702-5032</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Irvine CA</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>98</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>roofer Irvine CA</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>2026-10-07</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-07 21:25 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-07.xlsx
+++ b/output/leads_2026-10-07.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1508,6 +1508,62 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Residential Roofing Companies | Westminster, CO | UB Code Roofing +</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>ubcoderoofing.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://www.ubcoderoofing.com/contact/residential-roofing-companies-service-area/westminster-co</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>info@ubcoderoofing.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(303) 225-4620</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Westminster CO</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>residential roofing company Westminster CO</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>